<commit_message>
Map Data: Did more work on fishing
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98F340E-87D9-4213-BEF7-0BEB57C454A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DB147F-FDE5-4A06-AE51-063E21A41075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28800" windowHeight="17145" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="4635" yWindow="4635" windowWidth="28800" windowHeight="17145" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="100">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -269,6 +270,90 @@
   </si>
   <si>
     <t>Brawlzilla</t>
+  </si>
+  <si>
+    <t>Pokemon Dolls, Wishiwashi school sprite</t>
+  </si>
+  <si>
+    <t>SageDeoxys</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/sagedeoxys</t>
+  </si>
+  <si>
+    <t>MUST INFORM OF USE</t>
+  </si>
+  <si>
+    <t>Overworlds Of Sprigatito, Floragato, Meowscarada,  Fuecoco, Crocalor, Skeledirge, Quaxly, Quaxwell, Quaquaval, Lechonk, Oinkologne, Tarountula, Nymble, Lokix, Pawmi, Pawmo, Pawmot, Tandemaus, Maushold, Fidough, Dachsbun, Smoliv, Dolliv, Arboliva, Squawkabilly, Nacli, Naclstack, Garganacl, Charcadet, Armarouge, Ceruledge, Tadbulb, Bellibolt, Wattrel, Mabosstiff, Shroodle, Grafaiai, Bramblin, Brambleghast, Toedscool, Toedscruel, Klawf, Capsakid, Scovillain, Rellor, Rabsca, Flittle, Espathra, Tinkatink, Tinkatuff, Tinkaton, Wiglett, Wugtrio, Bombirdier, Finizen, Palafin, Cyclizar, Glimmet, Glimmora, Greavard, Houndstone, Flamigo, Cetoddle, Cetitan, Veluza,  Dodonzo, Tatsugiri, Orthworm, Clodsire, Farigiraf, Dudunsparce, Kingambit, Great Tusk, Scream Tail, Brute Bonnet, Flutter Mane, Slither Wing, Sandy Shocks, Iron Bundle, Iron Hands, Iron Treads, Iron Moth, Iron Thorns, Frigibax, Artibax, Baxcalibur, Gimmighoul, Gholdengo, Wo-Chien, Chien-Pao, Ting-Lu, Chi-Yu, Roaring Moon, Iron Valiant, Koraidon, Miraidon, Walking Wake, Iron Leaves, Dipplin, Poltchageist, Sinistcha, Munkidori, Fezandipiti, Ogerpon All Forms, Archaludon, Hydraapple, Gouging Fire, Raging Bolt, Iron Boulder, Iron Crown, Terapagos Normal form, Terapagos Terastal Form, Terapagos Stellar Form, Pecharunt Paldean Tauros, Paldean Wooper and Ursaluna Bloodmoon form by DarkusShadow</t>
+  </si>
+  <si>
+    <t>The Overworld of Spidops byEduarPokeN</t>
+  </si>
+  <si>
+    <t>Overworld of Maschiff and Annihilape by CarmaNekko</t>
+  </si>
+  <si>
+    <t>The Original Overworld of Iron Jugulis byTooManyLuigis, Mortedesu, Billla and Wolfang62</t>
+  </si>
+  <si>
+    <t>Original Slither Wing and Iron Moth Sprite byprincess-phoenix</t>
+  </si>
+  <si>
+    <t>Original Roaring Moon Sprite by Larryturbo</t>
+  </si>
+  <si>
+    <t>Original Brute Bonnet Sprite by TyranitarDark</t>
+  </si>
+  <si>
+    <t>Improved Koraidon's tail, antennae and face by shaderr31</t>
+  </si>
+  <si>
+    <t>Improvements in the colors of Dudunsparce, Tinkatink, Tinkatuff, and Tinkaton by Anarlaurendil</t>
+  </si>
+  <si>
+    <t>SS Anne And Sea Gallop</t>
+  </si>
+  <si>
+    <t>PeakyChew</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/peekychew/gallery</t>
+  </si>
+  <si>
+    <t>Custom House Set</t>
+  </si>
+  <si>
+    <t>WesleyFG</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/wesleyfg/art/PUBLIC-TILES-NOW-320643148</t>
+  </si>
+  <si>
+    <t>Aveontrainer</t>
+  </si>
+  <si>
+    <t>Bar Tileset, fossils, airplane, windmill, fishing hut</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/aveontrainer/gallery/68320549/tileset</t>
+  </si>
+  <si>
+    <t>TerribleJared</t>
+  </si>
+  <si>
+    <t>Boats and bike  sprites</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/terriblejared</t>
+  </si>
+  <si>
+    <t>Windmill</t>
+  </si>
+  <si>
+    <t>Anarlaurendil</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/anarlaurendil/art/Animated-windmill-sail-885505259</t>
   </si>
 </sst>
 </file>
@@ -313,7 +398,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -321,6 +406,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -657,7 +745,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.140625" bestFit="1" customWidth="1"/>
@@ -832,7 +920,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>57</v>
       </c>
@@ -843,7 +931,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -854,7 +942,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -865,7 +953,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -876,7 +964,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -887,7 +975,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -898,7 +986,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>59</v>
       </c>
@@ -909,7 +997,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>63</v>
       </c>
@@ -920,7 +1008,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>68</v>
       </c>
@@ -931,7 +1019,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -940,6 +1028,75 @@
       </c>
       <c r="C26" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>85</v>
+      </c>
+      <c r="B28" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" t="s">
+        <v>94</v>
+      </c>
+      <c r="C31" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -949,6 +1106,140 @@
     <hyperlink ref="B10" r:id="rId3" display="https://www.deviantart.com/thecubberx/gallery" xr:uid="{1CE16580-A4E8-4E2A-8B7A-6EEC4BA2FD45}"/>
     <hyperlink ref="B14" r:id="rId4" display="https://www.deviantart.com/aurumdeluxe" xr:uid="{DF54BD18-078B-4049-BEBB-106BDA490062}"/>
     <hyperlink ref="B19" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
+    <hyperlink ref="C30" r:id="rId6" xr:uid="{262F2778-6776-4F97-BB1B-C46A94C0844A}"/>
+    <hyperlink ref="B32" r:id="rId7" display="https://www.deviantart.com/anarlaurendil" xr:uid="{33DC61F5-9842-4EE8-B0F0-B653FB512E10}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3466180-0D67-48D9-B8A2-FCEB18F94623}">
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="223.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="90" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+    </row>
+    <row r="30" spans="1:1" ht="210" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1" display="https://www.deviantart.com/darkusshadow" xr:uid="{B7629F94-68A4-4C88-88F9-7BA8BD0E6188}"/>
+    <hyperlink ref="A5" r:id="rId2" display="https://www.deviantart.com/eduarpoken" xr:uid="{92477F86-EEF7-40DE-BE65-5E9930279B92}"/>
+    <hyperlink ref="A9" r:id="rId3" display="https://www.deviantart.com/carmanekko" xr:uid="{F5AD1522-3891-4DBE-8C76-27701753F0A5}"/>
+    <hyperlink ref="A13" r:id="rId4" display="https://www.deviantart.com/wolfang62" xr:uid="{AB9CAFF3-9135-4EBE-AB80-74250717C529}"/>
+    <hyperlink ref="A17" r:id="rId5" display="https://www.deviantart.com/princess-phoenix" xr:uid="{148A61A1-19D6-423E-806E-DB378563435A}"/>
+    <hyperlink ref="A21" r:id="rId6" display="https://www.deviantart.com/larryturbo" xr:uid="{A8FE2519-6A79-4EE5-820F-3F4ECC56F668}"/>
+    <hyperlink ref="A25" r:id="rId7" display="https://www.deviantart.com/tyranitardark" xr:uid="{50D00EFE-83B4-4076-AABF-7EBF3F2964A2}"/>
+    <hyperlink ref="A26" r:id="rId8" display="https://www.deviantart.com/shaderr31" xr:uid="{0E39BDA6-BB7F-4FF8-8E43-FD40B2FFBE1B}"/>
+    <hyperlink ref="A30" r:id="rId9" display="https://www.deviantart.com/anarlaurendil" xr:uid="{168EF457-0596-4D75-8C3F-1376B926BB22}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Map Data: Started adding missing extras and more buildings to Celeste Harbour
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DB147F-FDE5-4A06-AE51-063E21A41075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8D7BE7-8246-49C1-A25D-EBF3654470A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4635" yWindow="4635" windowWidth="28800" windowHeight="17145" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="106">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -354,6 +354,24 @@
   </si>
   <si>
     <t>https://www.deviantart.com/anarlaurendil/art/Animated-windmill-sail-885505259</t>
+  </si>
+  <si>
+    <t>Cresselia Plaza</t>
+  </si>
+  <si>
+    <t>Lapampa-fr</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/lapampa-fr/art/Cresselia-sanctuary-453250502</t>
+  </si>
+  <si>
+    <t>Darkness2118</t>
+  </si>
+  <si>
+    <t>Hoenn Style Moving Truck</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/darkness2118/art/BW-Style-Hoenn-Moving-Trucks-361814131</t>
   </si>
 </sst>
 </file>
@@ -745,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.140625" bestFit="1" customWidth="1"/>
@@ -1097,6 +1115,28 @@
       </c>
       <c r="C32" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>100</v>
+      </c>
+      <c r="B33" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>104</v>
+      </c>
+      <c r="B34" t="s">
+        <v>103</v>
+      </c>
+      <c r="C34" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fishing: Set up entirety of fish shop and fish storage
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8D7BE7-8246-49C1-A25D-EBF3654470A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6651544-0367-468E-97E4-16B54F622E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="112">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -372,6 +372,24 @@
   </si>
   <si>
     <t>https://www.deviantart.com/darkness2118/art/BW-Style-Hoenn-Moving-Trucks-361814131</t>
+  </si>
+  <si>
+    <t>Modern interiors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are Williarta </t>
+  </si>
+  <si>
+    <t>https://www.vecteezy.com/vector-art/82233938-pixel-art-ancient-scroll-illustration-for-retro-game-asset</t>
+  </si>
+  <si>
+    <t>Scroll</t>
+  </si>
+  <si>
+    <t>LimeZu</t>
+  </si>
+  <si>
+    <t>https://limezu.itch.io/moderninteriors</t>
   </si>
 </sst>
 </file>
@@ -763,7 +781,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.140625" bestFit="1" customWidth="1"/>
@@ -1139,6 +1157,28 @@
         <v>105</v>
       </c>
     </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" t="s">
+        <v>110</v>
+      </c>
+      <c r="C36" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="https://www.reddit.com/r/PokemonRMXP/" xr:uid="{484AF3F9-A79A-44A4-BE84-81893A8B5A0F}"/>
@@ -1148,6 +1188,7 @@
     <hyperlink ref="B19" r:id="rId5" display="https://www.deviantart.com/diegowt/gallery" xr:uid="{5595E6A6-D3C6-401E-81D5-305B7CA40024}"/>
     <hyperlink ref="C30" r:id="rId6" xr:uid="{262F2778-6776-4F97-BB1B-C46A94C0844A}"/>
     <hyperlink ref="B32" r:id="rId7" display="https://www.deviantart.com/anarlaurendil" xr:uid="{33DC61F5-9842-4EE8-B0F0-B653FB512E10}"/>
+    <hyperlink ref="B35" r:id="rId8" display="https://www.vecteezy.com/members/arewiliarta353003" xr:uid="{07D8F36A-6B1E-4035-9746-67EED19859B8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Card Data: GB card remakes and a few custom fan arts added
</commit_message>
<xml_diff>
--- a/Spreadsheets/credits.xlsx
+++ b/Spreadsheets/credits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FD2AF4-B405-413B-84FE-95432CE3BBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F5DC9F-4324-4C31-8C45-196BB9A03806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26115" yWindow="0" windowWidth="31590" windowHeight="15585" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{7635DB46-9F12-4EC4-9ABF-7C966C934E56}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="128">
   <si>
     <t>In Battle Trainer Sprites</t>
   </si>
@@ -399,6 +399,45 @@
   </si>
   <si>
     <t>Custom Ancient Latios, celebi, jirachi, uxie, crystal onix, chansey, blissey other custom cards</t>
+  </si>
+  <si>
+    <t>GB moltres zapdos articuno</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/linkinboss/gallery</t>
+  </si>
+  <si>
+    <t>Linkinboss</t>
+  </si>
+  <si>
+    <t>https://www.deviantart.com/katarawaterbender</t>
+  </si>
+  <si>
+    <t>Pokemon card template for custom cards</t>
+  </si>
+  <si>
+    <t>katarawaterbender</t>
+  </si>
+  <si>
+    <t>pansito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GB Ninetales, dragonite, pidgeot, vaporeon, jolteon, flareon, </t>
+  </si>
+  <si>
+    <t>GB illustration art (pidgeot)</t>
+  </si>
+  <si>
+    <t>GB card illustration art (vaporeon, jolteon, flareon)</t>
+  </si>
+  <si>
+    <t>turnip-miracle.tumblr.com/)</t>
+  </si>
+  <si>
+    <t>turnip-miracle</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/le.pansito/</t>
   </si>
 </sst>
 </file>
@@ -790,7 +829,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8449EA-7B8C-4284-BC16-D53892B08179}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="84.42578125" bestFit="1" customWidth="1"/>
@@ -1199,6 +1238,55 @@
         <v>112</v>
       </c>
     </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>122</v>
+      </c>
+      <c r="B39" t="s">
+        <v>117</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>119</v>
+      </c>
+      <c r="B40" t="s">
+        <v>120</v>
+      </c>
+      <c r="C40" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>124</v>
+      </c>
+      <c r="B41" t="s">
+        <v>121</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>123</v>
+      </c>
+      <c r="B42" t="s">
+        <v>126</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" display="https://www.reddit.com/r/PokemonRMXP/" xr:uid="{484AF3F9-A79A-44A4-BE84-81893A8B5A0F}"/>
@@ -1209,6 +1297,9 @@
     <hyperlink ref="C30" r:id="rId6" xr:uid="{262F2778-6776-4F97-BB1B-C46A94C0844A}"/>
     <hyperlink ref="B32" r:id="rId7" display="https://www.deviantart.com/anarlaurendil" xr:uid="{33DC61F5-9842-4EE8-B0F0-B653FB512E10}"/>
     <hyperlink ref="B35" r:id="rId8" display="https://www.vecteezy.com/members/arewiliarta353003" xr:uid="{07D8F36A-6B1E-4035-9746-67EED19859B8}"/>
+    <hyperlink ref="C42" r:id="rId9" display="https://www.deviantart.com/users/outgoing?http://turnip-miracle.tumblr.com/" xr:uid="{CD8CFDC0-8B02-4F38-8772-5F59BFB9801A}"/>
+    <hyperlink ref="C41" r:id="rId10" xr:uid="{F60B09CB-6997-4011-82F3-D10A7BFBA5E8}"/>
+    <hyperlink ref="C39" r:id="rId11" xr:uid="{BCBC95A3-D043-4247-A297-F8C99268C600}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>